<commit_message>
Title: Update element-to-work mapping logic to use partial text matching for level categories
Key features implemented:
- Modified `find_works_for_element` function to implement partial text matching when searching for corresponding work categories based on element level
- Updated level matching logic in `map_elements_to_works.py` to handle cases where element level strings like "до отм. 0,000" partially match longer work category strings like "Подземная часть здания (до ур. земли до отм. 0,000)"
- Adjusted `.gitignore` to include common Python build artifacts and Excel output files

The changes refine the mapping process to correctly associate elements with their corresponding work categories even when the naming conventions differ slightly between the element and work tables.
</commit_message>
<xml_diff>
--- a/uploads/4e073ac8-3a23-452a-b357-a822d29ae5fb/mapped_elements_works.xlsx
+++ b/uploads/4e073ac8-3a23-452a-b357-a822d29ae5fb/mapped_elements_works.xlsx
@@ -1,34 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,80 +45,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,14 +339,10 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>